<commit_message>
fix(lanzamiento): alinear Flujo Total y Tasa Crecimiento xlsx v3.8.2
Headers Año 1-5 en columnas D-H / C-G; I17=H17 activas cierre;
YoY revenue guard en fila 8; payback usa ABS($C$9). Regenera xlsx + verify.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Lanzamiento/MODELO_FINANCIERO_ZONIX_PHARMA.xlsx
+++ b/docs/Lanzamiento/MODELO_FINANCIERO_ZONIX_PHARMA.xlsx
@@ -3161,26 +3161,30 @@
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Año 1</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Año 2</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Año 2</t>
+          <t>Año 3</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Año 3</t>
+          <t>Año 4</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Año 4</t>
+          <t>Año 5</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -3216,7 +3220,7 @@
         <v/>
       </c>
       <c r="I17" s="7">
-        <f>N17</f>
+        <f>H17</f>
         <v/>
       </c>
     </row>
@@ -3578,7 +3582,7 @@
         </is>
       </c>
       <c r="C40" s="7">
-        <f>IF(H23&gt;=111988,5,IF(G23&gt;=111988,4,IF(F23&gt;=111988,3,IF(E23&gt;=111988,2,IF(D23&gt;=111988,1,"[LARGO PLAZO]")))))</f>
+        <f>IF(H23&gt;=ABS($C$9),5,IF(G23&gt;=ABS($C$9),4,IF(F23&gt;=ABS($C$9),3,IF(E23&gt;=ABS($C$9),2,IF(D23&gt;=ABS($C$9),1,"[LARGO PLAZO]")))))</f>
         <v/>
       </c>
     </row>
@@ -3600,7 +3604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I11"/>
+  <dimension ref="B2:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -3616,24 +3620,22 @@
           <t>Año 1</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Año 2</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Año 3</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Año 2</t>
+          <t>Año 4</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Año 3</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Año 4</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Año 5</t>
         </is>
@@ -3646,19 +3648,19 @@
         </is>
       </c>
       <c r="D6" s="9">
-        <f>IF(C7=0,"",(D8-C8)/C8)</f>
+        <f>IF(C8=0,"",(D8-C8)/C8)</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>IF(D7=0,"",(E8-D8)/D8)</f>
+        <f>IF(D8=0,"",(E8-D8)/D8)</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>IF(E7=0,"",(F8-E8)/E8)</f>
+        <f>IF(E8=0,"",(F8-E8)/E8)</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>IF(F7=0,"",(G8-F8)/F8)</f>
+        <f>IF(F8=0,"",(G8-F8)/F8)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(lanzamiento): alinear TIR a vector IRR columna J en Flujo Total
Las fórmulas TIR(3/5) apuntaban a K vacía mientras el vector vivía en J;
verify ahora valida J28=-SAFE y rango IRR(J…). Informe forense actualizado.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Lanzamiento/MODELO_FINANCIERO_ZONIX_PHARMA.xlsx
+++ b/docs/Lanzamiento/MODELO_FINANCIERO_ZONIX_PHARMA.xlsx
@@ -3560,7 +3560,7 @@
         </is>
       </c>
       <c r="C38" s="7">
-        <f>IRR(K28:K33)</f>
+        <f>IRR(J28:J33)</f>
         <v/>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
         </is>
       </c>
       <c r="C39" s="7">
-        <f>IRR(K28:K31)</f>
+        <f>IRR(J28:J31)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(lanzamiento): UX Flujo Total — TIR %, tasa r, resumen inversor Y5
Alinea legibilidad al template Pizza: Concepto B16, TIR con PCT_FMT, fila
Tasa Requerida (r), % SAFE recuperado, labels K22/L22; I17 vacío en activas.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Lanzamiento/MODELO_FINANCIERO_ZONIX_PHARMA.xlsx
+++ b/docs/Lanzamiento/MODELO_FINANCIERO_ZONIX_PHARMA.xlsx
@@ -3049,11 +3049,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:O42"/>
+  <dimension ref="B2:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3148,19 +3154,12 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>CCF</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>Por recuperar</t>
-        </is>
-      </c>
-    </row>
     <row r="16">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -3217,10 +3216,6 @@
       </c>
       <c r="H17" s="7">
         <f>'Año 5'!N11</f>
-        <v/>
-      </c>
-      <c r="I17" s="7">
-        <f>H17</f>
         <v/>
       </c>
     </row>
@@ -3377,6 +3372,16 @@
         <f>H20*$C$6</f>
         <v/>
       </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>CCF acum Y5</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Por recuperar Y5</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="6" t="inlineStr">
@@ -3559,7 +3564,7 @@
           <t>TIR(5)</t>
         </is>
       </c>
-      <c r="C38" s="7">
+      <c r="C38" s="9">
         <f>IRR(J28:J33)</f>
         <v/>
       </c>
@@ -3570,7 +3575,7 @@
           <t>TIR(3)</t>
         </is>
       </c>
-      <c r="C39" s="7">
+      <c r="C39" s="9">
         <f>IRR(J28:J31)</f>
         <v/>
       </c>
@@ -3578,16 +3583,49 @@
     <row r="40">
       <c r="B40" s="6" t="inlineStr">
         <is>
+          <t>Tasa Requerida (r)</t>
+        </is>
+      </c>
+      <c r="C40" s="9">
+        <f>$C$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="6" t="inlineStr">
+        <is>
           <t>Payback inversor (años, ilustrativo)</t>
         </is>
       </c>
-      <c r="C40" s="7">
+      <c r="C41" s="7">
         <f>IF(H23&gt;=ABS($C$9),5,IF(G23&gt;=ABS($C$9),4,IF(F23&gt;=ABS($C$9),3,IF(E23&gt;=ABS($C$9),2,IF(D23&gt;=ABS($C$9),1,"[LARGO PLAZO]")))))</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>% SAFE recuperado (CCF acum Y5, ilustrativo)</t>
+        </is>
+      </c>
+      <c r="C42" s="9">
+        <f>H23/ABS($C$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Lectura payback</t>
+        </is>
+      </c>
+      <c r="C43" s="7">
+        <f>IF(C41="[LARGO PLAZO]","CCF acum Y5 no cubre SAFE — ver % recuperado","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>NOTA: Reparto CCF/ECF ilustrativo post-cap SAFE 18,66%. No cláusula de dividendos.</t>
         </is>

</xml_diff>